<commit_message>
#206 mtd_schema_version を DbSpecifications.xlsx に追加する
- DbSpecifications.xlsx に mtd_schema_version を追加
</commit_message>
<xml_diff>
--- a/docs/DB/DbSpecifications.xlsx
+++ b/docs/DB/DbSpecifications.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26626"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Data\Program\C#\HouseholdAccountBook\db\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Data\Program\C#\HouseholdAccountBook\docs\DB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{078A0B3B-0A8B-4AE4-8E4D-AFD58F88E5A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D55A1CA2-3AF4-4F5B-A548-B64FF1EB1D2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" tabRatio="869" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7710" yWindow="3090" windowWidth="21600" windowHeight="11295" tabRatio="869" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="一覧" sheetId="1" r:id="rId1"/>
@@ -25,6 +25,8 @@
     <sheet name="備考(remark)" sheetId="4" r:id="rId10"/>
     <sheet name="Rel" sheetId="12" r:id="rId11"/>
     <sheet name="帳簿-項目(book_item)" sheetId="13" r:id="rId12"/>
+    <sheet name="Mtd" sheetId="14" r:id="rId13"/>
+    <sheet name="スキーマバージョン(schema_version)" sheetId="15" r:id="rId14"/>
   </sheets>
   <calcPr calcId="152511"/>
   <extLst>
@@ -36,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="219">
   <si>
     <t>テーブル論理名</t>
     <rPh sb="4" eb="7">
@@ -1155,6 +1157,33 @@
     </rPh>
     <rPh sb="31" eb="35">
       <t>ショウケンコウザ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>mtd_schema_version</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>version</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>バージョン</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>メタデータ</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>スキーマバージョン</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>PostgreSQLのみ。1行のみ</t>
+    <rPh sb="14" eb="15">
+      <t>ギョウ</t>
     </rPh>
     <phoneticPr fontId="1"/>
   </si>
@@ -1244,7 +1273,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1264,6 +1293,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1547,14 +1579,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:D10"/>
+  <dimension ref="B2:E11"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="2.875" customWidth="1"/>
-    <col min="2" max="3" width="14.25" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.25" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.15">
+    <row r="2" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1564,8 +1598,11 @@
       <c r="D2" s="1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.15">
+      <c r="E2" s="7" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="3" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B3" s="6" t="s">
         <v>3</v>
       </c>
@@ -1576,7 +1613,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="2:4" x14ac:dyDescent="0.15">
+    <row r="4" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B4" s="6" t="s">
         <v>6</v>
       </c>
@@ -1587,7 +1624,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="2:4" x14ac:dyDescent="0.15">
+    <row r="5" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B5" s="6" t="s">
         <v>188</v>
       </c>
@@ -1598,7 +1635,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="6" spans="2:4" x14ac:dyDescent="0.15">
+    <row r="6" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B6" s="6" t="s">
         <v>7</v>
       </c>
@@ -1609,7 +1646,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="2:4" x14ac:dyDescent="0.15">
+    <row r="7" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B7" s="6" t="s">
         <v>8</v>
       </c>
@@ -1620,7 +1657,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="2:4" x14ac:dyDescent="0.15">
+    <row r="8" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B8" s="6" t="s">
         <v>9</v>
       </c>
@@ -1631,7 +1668,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="2:4" x14ac:dyDescent="0.15">
+    <row r="9" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B9" s="6" t="s">
         <v>10</v>
       </c>
@@ -1642,7 +1679,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="2:4" x14ac:dyDescent="0.15">
+    <row r="10" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B10" s="6" t="s">
         <v>11</v>
       </c>
@@ -1651,6 +1688,20 @@
       </c>
       <c r="D10" t="s">
         <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B11" s="6" t="s">
+        <v>213</v>
+      </c>
+      <c r="C11" t="s">
+        <v>217</v>
+      </c>
+      <c r="D11" t="s">
+        <v>216</v>
+      </c>
+      <c r="E11" t="s">
+        <v>218</v>
       </c>
     </row>
   </sheetData>
@@ -1664,6 +1715,7 @@
     <hyperlink ref="B8" location="'分類(category)'!A1" display="mst_category" xr:uid="{00A03B14-0BD0-4A66-A7CE-342F682E6DB0}"/>
     <hyperlink ref="B9" location="'項目(item)'!A1" display="mst_item" xr:uid="{F48ABC00-5567-4F92-B80B-F0DBEC590B34}"/>
     <hyperlink ref="B10" location="'帳簿-項目(book_item)'!A1" display="rel_book_item" xr:uid="{B2D3E8FF-B862-4FAA-94EB-40D2A324AE47}"/>
+    <hyperlink ref="B11" location="'スキーマバージョン(schema_version)'!A1" display="mtd_schema_version" xr:uid="{47778E67-2115-4D13-8240-2CF2E5F64D9A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -2011,6 +2063,79 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4DFFCE8-02CD-4056-9269-7F14B944DE7B}">
+  <sheetPr>
+    <tabColor theme="5" tint="-0.249977111117893"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
+  <cols>
+    <col min="1" max="16384" width="9" style="2"/>
+  </cols>
+  <sheetData/>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD94830A-08C2-4E94-BBAC-7A3428F575EC}">
+  <dimension ref="B2:G4"/>
+  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
+  <cols>
+    <col min="2" max="2" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:7" x14ac:dyDescent="0.15">
+      <c r="B2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.15">
+      <c r="B3" t="s">
+        <v>215</v>
+      </c>
+      <c r="C3" t="s">
+        <v>214</v>
+      </c>
+      <c r="D3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" x14ac:dyDescent="0.15">
+      <c r="B4" t="s">
+        <v>73</v>
+      </c>
+      <c r="C4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>

</xml_diff>